<commit_message>
#3: doc: Technical information
</commit_message>
<xml_diff>
--- a/Doc/Bibliography/Models.xlsx
+++ b/Doc/Bibliography/Models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.marin\source\repos\arc-agi\Doc\Bibliography\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267C58AF-DF31-4708-ACC6-F35CA103F359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08288057-8BDF-488A-AED2-0834A4A62A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="67080" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,13 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="14">
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="16">
   <si>
     <t>Año</t>
   </si>
@@ -67,13 +61,25 @@
   </si>
   <si>
     <t>DSL</t>
+  </si>
+  <si>
+    <t>Precisión Total (FLOPS)</t>
+  </si>
+  <si>
+    <t>VRAM Total</t>
+  </si>
+  <si>
+    <t>Tiempo de entrenamiento (horas)</t>
+  </si>
+  <si>
+    <t>Coste por Token ($)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,8 +123,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -181,8 +203,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -242,23 +269,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -274,26 +317,32 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="8" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -307,33 +356,37 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="10" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="2" fontId="0" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="10" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="6" fillId="12" borderId="5" xfId="5" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="6">
     <cellStyle name="Bueno" xfId="1" builtinId="26"/>
+    <cellStyle name="Celda de comprobación" xfId="5" builtinId="23"/>
     <cellStyle name="Énfasis4" xfId="4" builtinId="41"/>
     <cellStyle name="Incorrecto" xfId="2" builtinId="27"/>
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
@@ -621,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.33203125" customWidth="1"/>
@@ -632,327 +685,374 @@
     <col min="6" max="6" width="25.77734375" customWidth="1"/>
     <col min="7" max="7" width="50.44140625" customWidth="1"/>
     <col min="8" max="8" width="25.88671875" customWidth="1"/>
-    <col min="9" max="9" width="44.77734375" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" customWidth="1"/>
+    <col min="10" max="10" width="23.21875" customWidth="1"/>
+    <col min="11" max="11" width="26.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>2020</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E2" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="25">
+      <c r="H2" s="32"/>
+      <c r="I2" s="25">
+        <v>2</v>
+      </c>
+      <c r="J2" s="25">
+        <v>9</v>
+      </c>
+      <c r="K2" s="32"/>
+    </row>
+    <row r="3" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="15">
         <v>2021</v>
       </c>
-      <c r="B3" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="27"/>
+      <c r="B3" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="17"/>
       <c r="D3" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="G3" s="17"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>2022</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
       <c r="D4" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G4" s="8"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="8"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>2023</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
       <c r="D5" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="11"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="16">
+        <v>10</v>
+      </c>
+      <c r="G5" s="10"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="18">
         <v>2024</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="14"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="14"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
+        <v>10</v>
+      </c>
+      <c r="G6" s="12"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="29"/>
+      <c r="K6" s="29"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="19"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="14"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
+        <v>10</v>
+      </c>
+      <c r="G7" s="12"/>
+      <c r="H7" s="29"/>
+      <c r="I7" s="29"/>
+      <c r="J7" s="29"/>
+      <c r="K7" s="29"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="19"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="14"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="14"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
+        <v>10</v>
+      </c>
+      <c r="G8" s="12"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
+      <c r="J8" s="29"/>
+      <c r="K8" s="29"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="19"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="14"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="14"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="17"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
+        <v>10</v>
+      </c>
+      <c r="G9" s="12"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="19"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="14"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="14"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="18"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
+        <v>10</v>
+      </c>
+      <c r="G10" s="12"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="29"/>
+      <c r="K10" s="29"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="20"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="14"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="14"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="19">
+        <v>10</v>
+      </c>
+      <c r="G11" s="12"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="29"/>
+      <c r="K11" s="29"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="21">
         <v>2025</v>
       </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
       <c r="D12" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="23"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="23"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="21"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+        <v>10</v>
+      </c>
+      <c r="G12" s="14"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="30"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="22"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
       <c r="D13" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="23"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="23"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="21"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+        <v>10</v>
+      </c>
+      <c r="G13" s="14"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
+      <c r="K13" s="30"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="22"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
       <c r="D14" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="23"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="23"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="21"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+        <v>10</v>
+      </c>
+      <c r="G14" s="14"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="30"/>
+      <c r="K14" s="30"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="22"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
       <c r="D15" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="23"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="23"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="21"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+        <v>10</v>
+      </c>
+      <c r="G15" s="14"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="30"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="22"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
       <c r="D16" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="23"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="23"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="22"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+        <v>10</v>
+      </c>
+      <c r="G16" s="14"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="23"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
       <c r="D17" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="23"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="23"/>
+        <v>10</v>
+      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C37" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>